<commit_message>
feat: add compact label print layout for 90x50mm sticker size
</commit_message>
<xml_diff>
--- a/三合一單網頁架機伺服器/地點代號對照表.xlsx
+++ b/三合一單網頁架機伺服器/地點代號對照表.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -788,6 +788,18 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>18P3A</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>EF180183A</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add PWA Dual-Track Architecture & Cloudflare D1 Backend
</commit_message>
<xml_diff>
--- a/三合一單網頁架機伺服器/地點代號對照表.xlsx
+++ b/三合一單網頁架機伺服器/地點代號對照表.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GOOGLE ANGET\三合一單自動產生器\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GOOGLE ANGET\三合一單網頁架機伺服器\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12135"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12132"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -27,9 +27,6 @@
     <t>長代號</t>
   </si>
   <si>
-    <t>預設料號</t>
-  </si>
-  <si>
     <t>彰濱二廠</t>
   </si>
   <si>
@@ -237,6 +234,10 @@
   </si>
   <si>
     <t>FAB7</t>
+  </si>
+  <si>
+    <t>預設料號</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -584,15 +585,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D34"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
-    <col min="2" max="2" width="14.42578125" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.625" customWidth="1"/>
+    <col min="2" max="2" width="14.375" customWidth="1"/>
+    <col min="3" max="3" width="11.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -600,352 +601,352 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>9</v>
       </c>
-      <c r="C5" t="s">
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" t="s">
+        <v>64</v>
+      </c>
+      <c r="D16" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" t="s">
+        <v>64</v>
+      </c>
+      <c r="D19" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>37</v>
+      </c>
+      <c r="B20" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" t="s">
+        <v>64</v>
+      </c>
+      <c r="D20" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" t="s">
+        <v>64</v>
+      </c>
+      <c r="D21" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" t="s">
+        <v>64</v>
+      </c>
+      <c r="D22" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" t="s">
+        <v>64</v>
+      </c>
+      <c r="D23" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>45</v>
+      </c>
+      <c r="B24" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" t="s">
+        <v>64</v>
+      </c>
+      <c r="D24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>47</v>
+      </c>
+      <c r="B25" t="s">
+        <v>48</v>
+      </c>
+      <c r="C25" t="s">
+        <v>64</v>
+      </c>
+      <c r="D25" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>57</v>
+      </c>
+      <c r="B30" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>59</v>
+      </c>
+      <c r="B31" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>61</v>
+      </c>
+      <c r="B32" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>63</v>
+      </c>
+      <c r="B33" t="s">
+        <v>38</v>
+      </c>
+      <c r="C33" t="s">
+        <v>64</v>
+      </c>
+      <c r="D33" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" t="s">
-        <v>65</v>
-      </c>
-      <c r="D14" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" t="s">
-        <v>29</v>
-      </c>
-      <c r="C15" t="s">
-        <v>65</v>
-      </c>
-      <c r="D15" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" t="s">
-        <v>31</v>
-      </c>
-      <c r="C16" t="s">
-        <v>65</v>
-      </c>
-      <c r="D16" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" t="s">
-        <v>35</v>
-      </c>
-      <c r="C18" t="s">
-        <v>65</v>
-      </c>
-      <c r="D18" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" t="s">
-        <v>65</v>
-      </c>
-      <c r="D19" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>38</v>
-      </c>
-      <c r="B20" t="s">
-        <v>39</v>
-      </c>
-      <c r="C20" t="s">
-        <v>65</v>
-      </c>
-      <c r="D20" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21" t="s">
-        <v>41</v>
-      </c>
-      <c r="C21" t="s">
-        <v>65</v>
-      </c>
-      <c r="D21" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" t="s">
-        <v>65</v>
-      </c>
-      <c r="D22" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>44</v>
-      </c>
-      <c r="B23" t="s">
-        <v>45</v>
-      </c>
-      <c r="C23" t="s">
-        <v>65</v>
-      </c>
-      <c r="D23" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>46</v>
-      </c>
-      <c r="B24" t="s">
-        <v>47</v>
-      </c>
-      <c r="C24" t="s">
-        <v>65</v>
-      </c>
-      <c r="D24" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>48</v>
-      </c>
-      <c r="B25" t="s">
-        <v>49</v>
-      </c>
-      <c r="C25" t="s">
-        <v>65</v>
-      </c>
-      <c r="D25" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>50</v>
-      </c>
-      <c r="B26" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>52</v>
-      </c>
-      <c r="B27" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>54</v>
-      </c>
-      <c r="B28" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>56</v>
-      </c>
-      <c r="B29" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>58</v>
-      </c>
-      <c r="B30" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>60</v>
-      </c>
-      <c r="B31" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>62</v>
-      </c>
-      <c r="B32" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>64</v>
-      </c>
-      <c r="B33" t="s">
-        <v>39</v>
-      </c>
-      <c r="C33" t="s">
-        <v>65</v>
-      </c>
-      <c r="D33" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>71</v>
-      </c>
       <c r="C34" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>